<commit_message>
Code tel qu'il fut lors de l'export final des configurations
</commit_message>
<xml_diff>
--- a/MATLAB/Optimisation/Optimisation REAR/optimisation_Hutchinson_plaque_transparente_finale/Rapports de configuration des plaques couvrantes/rapport de configuration plaque Hutchinson.xlsx
+++ b/MATLAB/Optimisation/Optimisation REAR/optimisation_Hutchinson_plaque_transparente_finale/Rapports de configuration des plaques couvrantes/rapport de configuration plaque Hutchinson.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucas.barbier\Documents\Maitrise dossier secondaire\MATLAB\Optimisation\Optimisation REAR\optimisation_Hutchinson_neutre_08_21_11_18\Rapports de configuration des plaques couvrantes\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucas.barbier\Documents\Maitrise dossier secondaire\MATLAB\Optimisation\Optimisation REAR\optimisation_Hutchinson_plaque_transparente_finale\Rapports de configuration des plaques couvrantes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{262D0943-E5FE-4B27-A933-27D23F021ED2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8084F3DC-0648-4ABA-8B9E-ED31E9F3A19D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1900" yWindow="1900" windowWidth="14400" windowHeight="7360" xr2:uid="{F684807A-0FE2-4E4B-9CB0-02CE5C3D1381}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{F684807A-0FE2-4E4B-9CB0-02CE5C3D1381}"/>
   </bookViews>
   <sheets>
     <sheet name="Paramètres globaux" sheetId="3" r:id="rId1"/>

</xml_diff>